<commit_message>
Improve dataset import and observation mapping
Add custom unit entry and larger previews, and let IC sets use mapped values from t=0 or the first data row.
</commit_message>
<xml_diff>
--- a/tests/data/synthetic/intermolecular_competition/M12_competition.xlsx
+++ b/tests/data/synthetic/intermolecular_competition/M12_competition.xlsx
@@ -7373,7 +7373,7 @@
         <v>0.95</v>
       </c>
       <c r="B98" s="4" t="n">
-        <v>78873832240.39551</v>
+        <v>50000000000.00005</v>
       </c>
       <c r="C98" s="5" t="n"/>
       <c r="D98" s="5" t="n"/>
@@ -7386,7 +7386,7 @@
         <v>0.96</v>
       </c>
       <c r="B99" s="4" t="n">
-        <v>511227717610.7139</v>
+        <v>40000000000.00004</v>
       </c>
       <c r="C99" s="5" t="n"/>
       <c r="D99" s="5" t="n"/>
@@ -7399,7 +7399,7 @@
         <v>0.97</v>
       </c>
       <c r="B100" s="4" t="n">
-        <v>5689233806286.617</v>
+        <v>30000000000.00003</v>
       </c>
       <c r="C100" s="5" t="n"/>
       <c r="D100" s="5" t="n"/>
@@ -7412,7 +7412,7 @@
         <v>0.98</v>
       </c>
       <c r="B101" s="4" t="n">
-        <v>169795925843960.9</v>
+        <v>20000000000.00002</v>
       </c>
       <c r="C101" s="5" t="n"/>
       <c r="D101" s="5" t="n"/>
@@ -7425,7 +7425,7 @@
         <v>0.99</v>
       </c>
       <c r="B102" s="4" t="n">
-        <v>5.639493994564991e+16</v>
+        <v>10000000000.00001</v>
       </c>
       <c r="C102" s="5" t="n"/>
       <c r="D102" s="5" t="n"/>

</xml_diff>